<commit_message>
feat: redesign general journal to management-oriented journal, implement operational source navigation (drill-down), and simplify manual entry creation
</commit_message>
<xml_diff>
--- a/public/templates/mau_so_du_dau_ky.xlsx
+++ b/public/templates/mau_so_du_dau_ky.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:N9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -419,9 +419,27 @@
         <v>Nguon tien</v>
       </c>
       <c r="G1" t="str">
+        <v>Kho</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Phong ban</v>
+      </c>
+      <c r="I1" t="str">
+        <v>So luong</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Don gia</v>
+      </c>
+      <c r="K1" t="str">
+        <v>So ky phan bo</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Ky bat dau phan bo</v>
+      </c>
+      <c r="M1" t="str">
         <v>So tien</v>
       </c>
-      <c r="H1" t="str">
+      <c r="N1" t="str">
         <v>Ghi chu</v>
       </c>
     </row>
@@ -444,10 +462,28 @@
       <c r="F2" t="str">
         <v>VCB_HCM</v>
       </c>
-      <c r="G2">
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2">
         <v>2500000000</v>
       </c>
-      <c r="H2" t="str">
+      <c r="N2" t="str">
         <v>So du ngan hang dau ky</v>
       </c>
     </row>
@@ -470,10 +506,28 @@
       <c r="F3" t="str">
         <v>TM_HCM</v>
       </c>
-      <c r="G3">
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3">
         <v>120000000</v>
       </c>
-      <c r="H3" t="str">
+      <c r="N3" t="str">
         <v>Quy tien mat dau ky</v>
       </c>
     </row>
@@ -496,10 +550,28 @@
       <c r="F4" t="str">
         <v/>
       </c>
-      <c r="G4">
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4">
         <v>50000000</v>
       </c>
-      <c r="H4" t="str">
+      <c r="N4" t="str">
         <v>Phai thu dau ky</v>
       </c>
     </row>
@@ -522,10 +594,28 @@
       <c r="F5" t="str">
         <v/>
       </c>
-      <c r="G5">
-        <v>-18500000</v>
+      <c r="G5" t="str">
+        <v/>
       </c>
       <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5">
+        <v>18500000</v>
+      </c>
+      <c r="N5" t="str">
         <v>Phai tra dau ky</v>
       </c>
     </row>
@@ -548,16 +638,166 @@
       <c r="F6" t="str">
         <v>VCB_HCM</v>
       </c>
-      <c r="G6">
-        <v>50000000</v>
+      <c r="G6" t="str">
+        <v/>
       </c>
       <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6">
+        <v>7000000</v>
+      </c>
+      <c r="N6" t="str">
         <v>Tien coc dang giu</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>2026-07</v>
+      </c>
+      <c r="B7" t="str">
+        <v>HCM</v>
+      </c>
+      <c r="C7" t="str">
+        <v>INVENTORY</v>
+      </c>
+      <c r="D7" t="str">
+        <v>NL001</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Nguyen lieu mau</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v>KHO_HCM</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7">
+        <v>50</v>
+      </c>
+      <c r="J7">
+        <v>32000</v>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7">
+        <v>1600000</v>
+      </c>
+      <c r="N7" t="str">
+        <v>Ton kho dau ky</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>2026-07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>HCM</v>
+      </c>
+      <c r="C8" t="str">
+        <v>ASSET</v>
+      </c>
+      <c r="D8" t="str">
+        <v>TS001</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Thiet bi dau ky</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v>STORE</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8">
+        <v>18000000</v>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8">
+        <v>18000000</v>
+      </c>
+      <c r="N8" t="str">
+        <v>Tai san/CCDC dau ky</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>2026-07</v>
+      </c>
+      <c r="B9" t="str">
+        <v>HCM</v>
+      </c>
+      <c r="C9" t="str">
+        <v>PREPAID_EXPENSE</v>
+      </c>
+      <c r="D9" t="str">
+        <v>PB001</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Chi phi phan bo dau ky</v>
+      </c>
+      <c r="F9" t="str">
+        <v>OPEX_RENT</v>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9">
+        <v>12</v>
+      </c>
+      <c r="L9" t="str">
+        <v>2026-07</v>
+      </c>
+      <c r="M9">
+        <v>120000000</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Chi phi phan bo dau ky</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(so-du-dau-ky): khai hạng mục P&L ngay khi nhập chi phí phân bổ
Khách phải chốt số dư rồi mở tab Trích trước gán lại hạng mục cho từng khoản thì số
phân bổ mới đứng đúng dòng P&L. Nay khai thẳng lúc nhập: form có ô Hạng mục P&L, file
import có cột cùng tên, cả hai đều không bắt buộc nhưng khai sai mã thì chặn ngay.

Hạng mục lưu trên bản ghi số dư (cột mới OpeningBalance.pnlItemCode), lúc chốt đi thẳng
sang khoản phân bổ nên bút toán 6428 hàng kỳ mang luôn mã hạng mục. currentAsInput cũng
phải mang theo cột này, nếu không lần PATCH đầu tiên xoá sạch giá trị vừa khai.

Kiểm chứng trên DB local qua API rồi xoá dữ liệu test: tạo số dư giữ đúng mã, chốt sinh
khoản PB-DK-* mang mã, ghi sổ ra Nợ 6428 kèm hạng mục / Có 242; mã sai bị chặn ở cả form
lẫn import; cột "Hang muc P&L" trên file Excel map đúng vào pnl_item_code.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/mau_so_du_dau_ky.xlsx
+++ b/public/templates/mau_so_du_dau_ky.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:O9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -437,9 +437,12 @@
         <v>Ky bat dau phan bo</v>
       </c>
       <c r="M1" t="str">
+        <v>Hang muc P&amp;L</v>
+      </c>
+      <c r="N1" t="str">
         <v>So tien</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>Ghi chu</v>
       </c>
     </row>
@@ -480,10 +483,13 @@
       <c r="L2" t="str">
         <v/>
       </c>
-      <c r="M2">
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2">
         <v>2500000000</v>
       </c>
-      <c r="N2" t="str">
+      <c r="O2" t="str">
         <v>So du ngan hang dau ky</v>
       </c>
     </row>
@@ -524,10 +530,13 @@
       <c r="L3" t="str">
         <v/>
       </c>
-      <c r="M3">
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3">
         <v>120000000</v>
       </c>
-      <c r="N3" t="str">
+      <c r="O3" t="str">
         <v>Quy tien mat dau ky</v>
       </c>
     </row>
@@ -568,10 +577,13 @@
       <c r="L4" t="str">
         <v/>
       </c>
-      <c r="M4">
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4">
         <v>50000000</v>
       </c>
-      <c r="N4" t="str">
+      <c r="O4" t="str">
         <v>Phai thu dau ky</v>
       </c>
     </row>
@@ -612,10 +624,13 @@
       <c r="L5" t="str">
         <v/>
       </c>
-      <c r="M5">
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5">
         <v>18500000</v>
       </c>
-      <c r="N5" t="str">
+      <c r="O5" t="str">
         <v>Phai tra dau ky</v>
       </c>
     </row>
@@ -656,10 +671,13 @@
       <c r="L6" t="str">
         <v/>
       </c>
-      <c r="M6">
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6">
         <v>7000000</v>
       </c>
-      <c r="N6" t="str">
+      <c r="O6" t="str">
         <v>Tien coc dang giu</v>
       </c>
     </row>
@@ -700,10 +718,13 @@
       <c r="L7" t="str">
         <v/>
       </c>
-      <c r="M7">
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7">
         <v>1600000</v>
       </c>
-      <c r="N7" t="str">
+      <c r="O7" t="str">
         <v>Ton kho dau ky</v>
       </c>
     </row>
@@ -744,10 +765,13 @@
       <c r="L8" t="str">
         <v/>
       </c>
-      <c r="M8">
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8">
         <v>18000000</v>
       </c>
-      <c r="N8" t="str">
+      <c r="O8" t="str">
         <v>Tai san/CCDC dau ky</v>
       </c>
     </row>
@@ -788,16 +812,19 @@
       <c r="L9" t="str">
         <v>2026-07</v>
       </c>
-      <c r="M9">
+      <c r="M9" t="str">
+        <v>PNL_THUE_MB</v>
+      </c>
+      <c r="N9">
         <v>120000000</v>
       </c>
-      <c r="N9" t="str">
+      <c r="O9" t="str">
         <v>Chi phi phan bo dau ky</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>